<commit_message>
Documents updated, crud service add new features, and update frontenf accordingly
</commit_message>
<xml_diff>
--- a/Documents/EXCEL TABLES/refund table.xlsx
+++ b/Documents/EXCEL TABLES/refund table.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project documents\EXCEL TABLES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,63 +24,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
-  <si>
-    <t>Column Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+  <si>
+    <t>Column no</t>
+  </si>
+  <si>
+    <t>Column name</t>
   </si>
   <si>
     <t>Data Type</t>
   </si>
   <si>
-    <t>Constraints</t>
-  </si>
-  <si>
-    <t>Default name</t>
+    <t>Constraint</t>
+  </si>
+  <si>
+    <t>Extra</t>
   </si>
   <si>
     <t>refund_id</t>
   </si>
   <si>
-    <t>PRIMARY KEY,AUTO_INCREMENT,NOT NULL</t>
+    <t>payment_id</t>
+  </si>
+  <si>
+    <t>ref_amount</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>refund_date</t>
   </si>
   <si>
     <t>int</t>
   </si>
   <si>
-    <t>payment_id</t>
-  </si>
-  <si>
-    <t>MULTIPLE,NOT NULL</t>
-  </si>
-  <si>
-    <t>refund_amount</t>
-  </si>
-  <si>
     <t>decimal(10,2)</t>
   </si>
   <si>
-    <t>refund_reason</t>
-  </si>
-  <si>
     <t>text</t>
   </si>
   <si>
-    <t>refund_status</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>refund_date</t>
-  </si>
-  <si>
     <t>timestamp</t>
   </si>
   <si>
-    <t>CURRENT_TIMESTAMP</t>
-  </si>
-  <si>
-    <t>enum('Pending','Processed','Rejected','Completed')</t>
+    <t>Primary Key</t>
+  </si>
+  <si>
+    <t>auto_incemented</t>
+  </si>
+  <si>
+    <t>Foreign key</t>
+  </si>
+  <si>
+    <t>current_timestamp</t>
   </si>
 </sst>
 </file>
@@ -398,16 +395,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:D9"/>
+  <dimension ref="A2:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="46.85546875" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" customWidth="1"/>
-    <col min="4" max="4" width="20.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="21.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -420,64 +418,74 @@
       <c r="D2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="E8" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>